<commit_message>
docs: AI B independent verification (10/10 PASS, offline-dom + real http-server)
</commit_message>
<xml_diff>
--- a/T05_AI_REQUEST_LOG_v1.0.0.xlsx
+++ b/T05_AI_REQUEST_LOG_v1.0.0.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -660,7 +660,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -681,6 +681,12 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1188,7 +1194,7 @@
       <c r="C5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>46292.67872685185</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1275,13 +1281,15 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Claude / 실제 사용 모델 기록</t>
+          <t>Claude (Anthropic) / Claude Sonnet 5 (claude-sonnet-5; 채팅 인터페이스 표시명, 백엔드 버전 ID는 독립 미확인)</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="5" t="str"/>
+      <c r="D10" s="11" t="n">
+        <v>46292.70069444444</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>이 프로젝트는 다른 AI가 먼저 작업한 상태입니다. 이전 AI와의 대화 내용은 제공하지 않습니다.
@@ -1293,7 +1301,14 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>최초 요청</t>
+          <t>요청 1/5회차
+인수인계 상태 확인: HANDOFF.md 종료 소스 커밋 5cc2ac4e9a203c71cab049fa2d1f4e79dc8b2093 및 문서화 커밋 1c3a36ec8ae242e454f7266fc22351101bfac41a 확인. finalize_handoff.py 재실행 결과 '이미 반영됨'.
+B 시작 HEAD: 1c3a36ec8ae242e454f7266fc22351101bfac41a
+실행: tools/verify-official-assets.py -&gt; 17개 전부 OK.
+실행: tools/test_t05.py --offline-dom --actor AI_B -&gt; TEST-01~10 10/10 PASS, 보조 검증 8건 전부 PASS.
+실행: tools/test_t05.py --actor AI_B (실제 http.server, mocked 외부 API route, 네이티브 localStorage) -&gt; TEST-01~10 10/10 PASS, 보조 검증 7건 전부 PASS(오프라인 전용 항목 1건 자동 제외).
+재현되는 기능 결함 없음. 애플리케이션 소스(index.html/script.js/style.css) 변경 없음.
+시각: 도구 관측값(KST) 기준, 정확한 채팅 전달 시각은 미확인. 세부는 T05_RESULT.md 참조.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: AI B request 2/5 - fill request log and working-time record
</commit_message>
<xml_diff>
--- a/T05_AI_REQUEST_LOG_v1.0.0.xlsx
+++ b/T05_AI_REQUEST_LOG_v1.0.0.xlsx
@@ -1318,13 +1318,43 @@
           <t>AI B</t>
         </is>
       </c>
-      <c r="B11" s="5" t="str"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Claude (Anthropic) / Claude Sonnet 5 (claude-sonnet-5; 채팅 인터페이스 표시명, 백엔드 버전 ID는 독립 미확인)</t>
+        </is>
+      </c>
       <c r="C11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="5" t="str"/>
-      <c r="E11" s="5" t="str"/>
-      <c r="F11" s="5" t="str"/>
+      <c r="D11" s="11" t="n">
+        <v>46292.71736111111</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>이 요청은 AI B의 요청 2/5회차입니다.
+새로운 기능을 추가하거나 애플리케이션 소스를 수정하지 말고, 방금 완료한 AI B 작업의 기록 누락만 보완해 주세요.
+1. T05_AI_REQUEST_LOG_v1.0.0.xlsx의 AI B 2회차에 이번 요청의 요청 일시, 요청 원문, 처리 결과를 기록해 주세요.
+2. T05_RESULT.md에 AI B의 작업시간 기록을 보완해 주세요.
+- 시작 시각은 기존 요청 기록의 2026-09-27 16:49:00 KST를 사용합니다.
+- 종료 시각은 이번 최종 결과를 전달하기 직전에 실제로 확인 가능한 KST 시각을 기록해 주세요.
+- 시작 시각과 종료 시각을 기준으로 실제 작업시간을 계산해 주세요.
+- 확인하지 못한 시각을 추측해서 작성하지 마세요.
+3. T05_RESULT.md 상단에 남아 있는 "AI B와 최종 비교는 아직 실행하지 않았습니다." 문구는 현재 B 작업 완료 상태에 맞게 수정해 주세요.
+4. 기존 AI A 기록과 검사 이력은 변경하지 마세요.
+5. 다음 파일과 기준은 변경하지 마세요: index.html, style.css, script.js, T05_EXPERIMENT_PLAN.md, HANDOFF.md, TEST-01~TEST-10의 입력 및 기대값, 기존 AI A 요청 기록 및 evidence.
+6. 기존 AI B의 검사 결과와 커밋 이력도 삭제하지 말고 그대로 보존해 주세요.
+작업을 마친 뒤 변경 사항을 커밋하고, 새 Full Commit ID / 갱신된 T05_AI_REQUEST_LOG_v1.0.0.xlsx / 갱신된 T05_RESULT.md / 최종 프로젝트 ZIP을 제공해 주세요.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>요청 2/5회차. 애플리케이션 소스(index.html/script.js/style.css)와 T05_EXPERIMENT_PLAN.md/HANDOFF.md/TEST-01~10/AI A 기록·evidence는 변경하지 않았습니다.
+T05_AI_REQUEST_LOG_v1.0.0.xlsx AI B 2회차(이 행) 기록.
+T05_RESULT.md에 AI B 작업시간(시작 2026-09-27 16:49 KST, 종료 2026-09-27 17:13 KST, 실제 작업시간 24분) 보완, 상단 안내 문구를 B 완료 상태로 수정.
+기존 AI B 커밋(58533c7, a9820eb) 및 A 기록/검사 이력은 삭제·수정 없이 그대로 보존.
+요청 일시는 이번 응답 전달 직전 확인한 도구 관측값(KST)이며, 정확한 채팅 전달 시각은 미확인입니다.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: finalize T05 experiment records
</commit_message>
<xml_diff>
--- a/T05_AI_REQUEST_LOG_v1.0.0.xlsx
+++ b/T05_AI_REQUEST_LOG_v1.0.0.xlsx
@@ -1180,7 +1180,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="210" customHeight="1">
+    <row r="5" ht="235" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>AI A</t>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ChatGPT / GPT-6 Astra Pro</t>
+          <t>ChatGPT / GPT-5.6 Sol</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -1213,7 +1213,8 @@
 고정 환율 + 오프라인 DOM 검증
 실제 배포·라이브 조회: 미확인
 시각: 시작 직후 도구 관측값(KST). 정확한 전송 시각 미확인.
-오류·중단 기록, 종료 관측시각은 T05_RESULT.md 참조.</t>
+오류·중단 기록, 종료 관측시각은 T05_RESULT.md 참조.
+기록 정정: 초기 산출물의 AI A 모델명 오기를 실제 모델 GPT-5.6 Sol로 정정. 요청 원문·시각·검사 결과는 변경하지 않음.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1274,7 @@
       <c r="E9" s="5" t="str"/>
       <c r="F9" s="5" t="str"/>
     </row>
-    <row r="10" ht="140" customHeight="1">
+    <row r="10" ht="260" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>AI B</t>
@@ -1312,7 +1313,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="330" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>AI B</t>
@@ -1326,8 +1327,10 @@
       <c r="C11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="11" t="n">
-        <v>46292.71736111111</v>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -1352,7 +1355,8 @@
 T05_AI_REQUEST_LOG_v1.0.0.xlsx AI B 2회차(이 행) 기록.
 T05_RESULT.md에 AI B 작업시간(시작 2026-09-27 16:49 KST, 종료 2026-09-27 17:13 KST, 실제 작업시간 24분) 보완, 상단 안내 문구를 B 완료 상태로 수정.
 기존 AI B 커밋(58533c7, a9820eb) 및 A 기록/검사 이력은 삭제·수정 없이 그대로 보존.
-요청 일시는 이번 응답 전달 직전 확인한 도구 관측값(KST)이며, 정확한 채팅 전달 시각은 미확인입니다.</t>
+요청 일시는 이번 응답 전달 직전 확인한 도구 관측값(KST)이며, 정확한 채팅 전달 시각은 미확인입니다.
+시각 정정: 정확한 2회차 요청 수신 시각은 확인할 수 없어 요청 일시는 미확인으로 둠. 2026-09-27 17:13 KST는 응답 전달 직전 도구 관측값이며 T05_RESULT.md의 종료 시각 근거로만 사용.</t>
         </is>
       </c>
     </row>

</xml_diff>